<commit_message>
BusTickets feature file added
</commit_message>
<xml_diff>
--- a/SeleniumUIFramework.RedbusApp/src/test/resources/Readers/Config.xlsx
+++ b/SeleniumUIFramework.RedbusApp/src/test/resources/Readers/Config.xlsx
@@ -1,21 +1,17 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27932"/>
-  <workbookPr defaultThemeVersion="202300"/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\sivap\Downloads\"/>
-    </mc:Choice>
-  </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{5139C15A-E00D-40A2-9BDA-963EB61DBEDD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
+  <workbookPr/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:801_{CAD43681-E264-4E17-9E9F-F1B139689CEB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{7104D9CB-5453-4DB5-8EE8-3184285F4ED3}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{7104D9CB-5453-4DB5-8EE8-3184285F4ED3}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="191029"/>
+  <calcPr calcId="0"/>
+  <oleSize ref="A1"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -27,15 +23,14 @@
         <xcalcf:feature name="microsoft.com:FV"/>
         <xcalcf:feature name="microsoft.com:CNMTM"/>
         <xcalcf:feature name="microsoft.com:LET_WF"/>
-        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
-        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
       </xcalcf:calcFeatures>
-    </ext>
-    <ext xmlns:xlwcv="http://schemas.microsoft.com/office/spreadsheetml/2024/workbookCompatibilityVersion" uri="{D14903EA-33C4-47F7-8F05-3474C54BE107}">
-      <xlwcv:version setVersion="1"/>
     </ext>
   </extLst>
 </workbook>
+</file>
+
+<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
@@ -407,7 +402,9 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9268388E-28BE-441C-B6D1-8CB9C41A57A5}">
   <dimension ref="A1"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
-  <sheetData/>
+  <sheetData>
+    <row r="1" spans="1:1" x14ac:dyDescent="0.3"/>
+  </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>